<commit_message>
Made it so all data now gets pulled from a local csv file and filled into the html
</commit_message>
<xml_diff>
--- a/Coin Data.xlsx
+++ b/Coin Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\coin-flips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D1C41C0-F7F8-4BBB-AD71-B59271044D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C4FF0C-3816-4B23-864E-501E898702CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="3225" windowWidth="28800" windowHeight="15435" xr2:uid="{9E5DD61D-E2DC-4DDF-B1A0-ED9C8FE585C6}"/>
+    <workbookView xWindow="4275" yWindow="2130" windowWidth="28800" windowHeight="15435" xr2:uid="{9E5DD61D-E2DC-4DDF-B1A0-ED9C8FE585C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Coin Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
   <si>
     <t>Flip</t>
   </si>
@@ -52,9 +52,6 @@
     <t>ID</t>
   </si>
   <si>
-    <t>1, 1</t>
-  </si>
-  <si>
     <t>20.5mm</t>
   </si>
   <si>
@@ -70,56 +67,68 @@
     <t>Lincoln Bicentennial</t>
   </si>
   <si>
-    <t>1, 2</t>
-  </si>
-  <si>
     <t>P</t>
   </si>
   <si>
     <t>Presidency</t>
   </si>
   <si>
-    <t>1, 3</t>
-  </si>
-  <si>
     <t>Childhood</t>
   </si>
   <si>
-    <t>2, 1</t>
-  </si>
-  <si>
-    <t>2, 2</t>
-  </si>
-  <si>
     <t>Formative Years</t>
   </si>
   <si>
-    <t>2, 3</t>
-  </si>
-  <si>
-    <t>3, 1</t>
-  </si>
-  <si>
-    <t>3, 2</t>
-  </si>
-  <si>
-    <t>3, 3</t>
-  </si>
-  <si>
-    <t>4, 1</t>
-  </si>
-  <si>
-    <t>4, 2</t>
-  </si>
-  <si>
-    <t>4, 3</t>
+    <t>1-1</t>
+  </si>
+  <si>
+    <t>1-2</t>
+  </si>
+  <si>
+    <t>1-3</t>
+  </si>
+  <si>
+    <t>2-1</t>
+  </si>
+  <si>
+    <t>2-2</t>
+  </si>
+  <si>
+    <t>2-3</t>
+  </si>
+  <si>
+    <t>3-1</t>
+  </si>
+  <si>
+    <t>3-2</t>
+  </si>
+  <si>
+    <t>3-3</t>
+  </si>
+  <si>
+    <t>4-1</t>
+  </si>
+  <si>
+    <t>4-2</t>
+  </si>
+  <si>
+    <t>4-3</t>
+  </si>
+  <si>
+    <t>2005</t>
+  </si>
+  <si>
+    <t>Lincoln Cent</t>
+  </si>
+  <si>
+    <t>999</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -596,8 +605,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -974,253 +984,318 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A309B3-79F7-41B9-B68C-B59FE202E6B3}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="21.140625" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="16.75" customWidth="1"/>
-    <col min="9" max="9" width="20.125" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2">
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1">
         <v>2009</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="G3" s="1"/>
+      <c r="H3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J3" s="1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
+        <v>2009</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J2">
-        <v>46</v>
+      <c r="F4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="1">
+        <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1">
+        <v>2009</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D3">
+      <c r="F5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1">
         <v>2009</v>
       </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="E6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3">
-        <v>47</v>
+      <c r="I6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="1">
+        <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1">
+        <v>2009</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4">
+      <c r="F7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1">
         <v>2009</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4">
-        <v>44</v>
-      </c>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
     </row>
-    <row r="5" spans="1:10">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>2009</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5">
-        <v>45</v>
-      </c>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
     </row>
-    <row r="6" spans="1:10">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>2009</v>
-      </c>
-      <c r="E6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6">
-        <v>48</v>
-      </c>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
     </row>
-    <row r="7" spans="1:10">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7">
-        <v>2009</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7">
-        <v>49</v>
-      </c>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
     </row>
-    <row r="8" spans="1:10">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8">
-        <v>2009</v>
-      </c>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
     </row>
-    <row r="9" spans="1:10">
-      <c r="A9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" t="s">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B13" t="s">
-        <v>11</v>
-      </c>
+      <c r="B13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Now dynamically sets the coin size via javascript and css properties!
</commit_message>
<xml_diff>
--- a/Coin Data.xlsx
+++ b/Coin Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\coin-flips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C4FF0C-3816-4B23-864E-501E898702CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA6470A-9B7E-491B-8A86-C85AE7192465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="2130" windowWidth="28800" windowHeight="15435" xr2:uid="{9E5DD61D-E2DC-4DDF-B1A0-ED9C8FE585C6}"/>
+    <workbookView xWindow="3360" yWindow="2070" windowWidth="28800" windowHeight="15435" xr2:uid="{9E5DD61D-E2DC-4DDF-B1A0-ED9C8FE585C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Coin Data" sheetId="1" r:id="rId1"/>
@@ -20,14 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="37">
   <si>
     <t>Flip</t>
   </si>
   <si>
-    <t>Flip Size</t>
-  </si>
-  <si>
     <t>Top Note</t>
   </si>
   <si>
@@ -122,6 +119,18 @@
   </si>
   <si>
     <t>999</t>
+  </si>
+  <si>
+    <t>Window Size</t>
+  </si>
+  <si>
+    <t>20mm</t>
+  </si>
+  <si>
+    <t>10mm</t>
+  </si>
+  <si>
+    <t>40mm</t>
   </si>
 </sst>
 </file>
@@ -997,88 +1006,88 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1">
         <v>2009</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J3" s="1">
         <v>47</v>
@@ -1086,27 +1095,27 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1">
         <v>2009</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J4" s="1">
         <v>44</v>
@@ -1114,27 +1123,27 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1">
         <v>2009</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5" s="1">
         <v>45</v>
@@ -1142,27 +1151,27 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1">
         <v>2009</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J6" s="1">
         <v>48</v>
@@ -1170,27 +1179,27 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1">
         <v>2009</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J7" s="1">
         <v>49</v>
@@ -1198,10 +1207,10 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1">
@@ -1216,10 +1225,10 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1232,10 +1241,10 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1248,10 +1257,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1264,10 +1273,10 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1280,10 +1289,10 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>

</xml_diff>

<commit_message>
Added a guide option in the excel sheet and made guides turn off when that option is choosed
</commit_message>
<xml_diff>
--- a/Coin Data.xlsx
+++ b/Coin Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\coin-flips\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA6470A-9B7E-491B-8A86-C85AE7192465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5628E2FE-1B1F-4C19-9978-B9E49C6F15D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3360" yWindow="2070" windowWidth="28800" windowHeight="15435" xr2:uid="{9E5DD61D-E2DC-4DDF-B1A0-ED9C8FE585C6}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="36">
   <si>
     <t>Flip</t>
   </si>
@@ -124,13 +124,10 @@
     <t>Window Size</t>
   </si>
   <si>
-    <t>20mm</t>
-  </si>
-  <si>
-    <t>10mm</t>
-  </si>
-  <si>
-    <t>40mm</t>
+    <t>Guideline</t>
+  </si>
+  <si>
+    <t>off</t>
   </si>
 </sst>
 </file>
@@ -992,318 +989,394 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A309B3-79F7-41B9-B68C-B59FE202E6B3}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="21.140625" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
+      <c r="K1" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>32</v>
+      <c r="K2" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1">
+        <v>31</v>
+      </c>
+      <c r="C3" s="1">
         <v>2009</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="1">
+      <c r="I3" s="1">
         <v>47</v>
       </c>
+      <c r="J3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2009</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="1">
+        <v>44</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1">
-        <v>2009</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="1">
-        <v>44</v>
+      <c r="K4" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2009</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="1">
+        <v>45</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1">
-        <v>2009</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J5" s="1">
-        <v>45</v>
+      <c r="K5" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2009</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" s="1">
+        <v>48</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1">
-        <v>2009</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="1">
-        <v>48</v>
-      </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2009</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="1">
+        <v>49</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1">
-        <v>2009</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J7" s="1">
-        <v>49</v>
+      <c r="K7" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1">
         <v>2009</v>
       </c>
-      <c r="E8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
+      <c r="J9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
+      <c r="J10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="E11" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
+      <c r="J12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="E13" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
+      <c r="J13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K13" xr:uid="{2475A098-2E8E-490B-A264-66E36B505B9D}">
+      <formula1>"off, on"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>